<commit_message>
Create a SimManager workflow for UC mapping from surrogate-input to full A1 models
</commit_message>
<xml_diff>
--- a/test_data/main/test_subnet_opt_A1/rate_cmp.xlsx
+++ b/test_data/main/test_subnet_opt_A1/rate_cmp.xlsx
@@ -1,29 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\Salvador\repo\model_tuner\test_data\main\test_subnet_opt_A1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75D0C57C-4CD2-47BB-86E7-9AD9B17C0328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B021CDE-D6CB-484D-89E4-26E2638442F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{FDB89A72-0890-442E-8838-6901716639C3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="4" xr2:uid="{FDB89A72-0890-442E-8838-6901716639C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
     <sheet name="wmult=0.02" sheetId="2" r:id="rId2"/>
     <sheet name="Лист2" sheetId="3" r:id="rId3"/>
     <sheet name="Лист3" sheetId="9" r:id="rId4"/>
-    <sheet name="wmult_0.02_pyr_pv_3s_1" sheetId="6" r:id="rId5"/>
-    <sheet name="wmult_0.05_pyr_pv_5s_ramp" sheetId="8" r:id="rId6"/>
-    <sheet name="Лист4" sheetId="7" r:id="rId7"/>
+    <sheet name="Лист5" sheetId="10" r:id="rId5"/>
+    <sheet name="wmult_0.02_pyr_pv_3s_1" sheetId="6" r:id="rId6"/>
+    <sheet name="wmult_0.05_pyr_pv_5s_ramp" sheetId="8" r:id="rId7"/>
+    <sheet name="Лист4" sheetId="7" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="4" hidden="1">wmult_0.02_pyr_pv_3s_1!$A$1:$BK$44</definedName>
-    <definedName name="ExternalData_1" localSheetId="5" hidden="1">wmult_0.05_pyr_pv_5s_ramp!$A$1:$BK$44</definedName>
+    <definedName name="ExternalData_1" localSheetId="5" hidden="1">wmult_0.02_pyr_pv_3s_1!$A$1:$BK$44</definedName>
+    <definedName name="ExternalData_1" localSheetId="6" hidden="1">wmult_0.05_pyr_pv_5s_ramp!$A$1:$BK$44</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6244" uniqueCount="927">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6283" uniqueCount="938">
   <si>
     <t xml:space="preserve">   SOM5Bfrz : 5.241 Hz</t>
   </si>
@@ -2830,6 +2831,40 @@
   </si>
   <si>
     <t>i_ou_wmult=0.02_10s</t>
+  </si>
+  <si>
+    <t>1_unconn</t>
+  </si>
+  <si>
+    <t>5_IT_PV_noramp_10s</t>
+  </si>
+  <si>
+    <t>6_IT_PV_ramp_10s</t>
+  </si>
+  <si>
+    <t>4_PYR_PV_noramp</t>
+  </si>
+  <si>
+    <t>2_PYR_PV_ramp</t>
+  </si>
+  <si>
+    <t>7_SELF_ramp</t>
+  </si>
+  <si>
+    <t>8_SELF_noramp</t>
+  </si>
+  <si>
+    <t>9_SELF_CON_TO_SUR_noramp</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>(PV6 slow osc.)
+try sur_to_con</t>
+  </si>
+  <si>
+    <t>try unconn + ramp</t>
   </si>
 </sst>
 </file>
@@ -2853,7 +2888,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2878,6 +2913,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -2891,7 +2938,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -2903,6 +2950,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -6674,6 +6733,773 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AE0FE40-67D7-40A0-A459-56D7A9322B1E}">
+  <dimension ref="B1:P28"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="17.109375" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" style="4"/>
+    <col min="4" max="4" width="9.5546875" style="4" customWidth="1"/>
+    <col min="5" max="5" width="11" style="4" customWidth="1"/>
+    <col min="6" max="6" width="17.33203125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="19.77734375" style="4" customWidth="1"/>
+    <col min="8" max="8" width="17.77734375" style="4" customWidth="1"/>
+    <col min="9" max="9" width="19.44140625" style="4" customWidth="1"/>
+    <col min="10" max="10" width="17.6640625" style="4" customWidth="1"/>
+    <col min="11" max="11" width="15.44140625" style="4" customWidth="1"/>
+    <col min="12" max="12" width="8.88671875" style="4"/>
+    <col min="13" max="13" width="28.109375" style="4" customWidth="1"/>
+    <col min="14" max="16" width="8.88671875" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="D1" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>927</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>931</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>929</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>930</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>928</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>932</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>933</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C3" s="4" t="s">
+        <v>557</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="E3" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0.08</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0.15</v>
+      </c>
+      <c r="H3" s="5">
+        <v>30.31</v>
+      </c>
+      <c r="I3" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="J3" s="4">
+        <v>0.08</v>
+      </c>
+      <c r="K3" s="4">
+        <v>0.08</v>
+      </c>
+      <c r="M3" s="4">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="4" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C4" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="D4" s="4">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="E4" s="4">
+        <v>9.5399999999999991</v>
+      </c>
+      <c r="F4" s="7">
+        <v>5.62</v>
+      </c>
+      <c r="G4" s="4">
+        <v>9.3800000000000008</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4">
+        <v>8.85</v>
+      </c>
+      <c r="J4" s="4">
+        <v>9.6199999999999992</v>
+      </c>
+      <c r="K4" s="4">
+        <v>11.62</v>
+      </c>
+      <c r="M4" s="4">
+        <v>7.08</v>
+      </c>
+    </row>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C5" s="4" t="s">
+        <v>568</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0.06</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="H5" s="5">
+        <v>29.78</v>
+      </c>
+      <c r="I5" s="5">
+        <v>32.49</v>
+      </c>
+      <c r="J5" s="4">
+        <v>0.06</v>
+      </c>
+      <c r="K5" s="5">
+        <v>32.28</v>
+      </c>
+      <c r="M5" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C6" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="D6" s="4">
+        <v>9.6</v>
+      </c>
+      <c r="E6" s="4">
+        <v>11.01</v>
+      </c>
+      <c r="F6" s="7">
+        <v>6.06</v>
+      </c>
+      <c r="G6" s="4">
+        <v>7.24</v>
+      </c>
+      <c r="H6" s="10">
+        <v>0</v>
+      </c>
+      <c r="I6" s="10">
+        <v>0</v>
+      </c>
+      <c r="J6" s="4">
+        <v>9.8800000000000008</v>
+      </c>
+      <c r="K6" s="4">
+        <v>11.77</v>
+      </c>
+      <c r="M6" s="4">
+        <v>10.029999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C7" s="4" t="s">
+        <v>594</v>
+      </c>
+      <c r="D7" s="4">
+        <v>2.1</v>
+      </c>
+      <c r="E7" s="8">
+        <v>0.96</v>
+      </c>
+      <c r="F7" s="5">
+        <v>0.02</v>
+      </c>
+      <c r="G7" s="5">
+        <v>0.26</v>
+      </c>
+      <c r="H7" s="5">
+        <v>21.41</v>
+      </c>
+      <c r="I7" s="5">
+        <v>7.73</v>
+      </c>
+      <c r="J7" s="5">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="K7" s="5">
+        <v>10.33</v>
+      </c>
+      <c r="M7" s="4">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B8" t="s">
+        <v>937</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="D8" s="4">
+        <v>10.1</v>
+      </c>
+      <c r="E8" s="4">
+        <v>12.85</v>
+      </c>
+      <c r="F8" s="10">
+        <v>0</v>
+      </c>
+      <c r="G8" s="10">
+        <v>0.18</v>
+      </c>
+      <c r="H8" s="5">
+        <v>281.32</v>
+      </c>
+      <c r="I8" s="5">
+        <v>111.51</v>
+      </c>
+      <c r="J8" s="4">
+        <v>12.97</v>
+      </c>
+      <c r="K8" s="4">
+        <v>11.85</v>
+      </c>
+      <c r="M8" s="4">
+        <v>11.84</v>
+      </c>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C9" s="4" t="s">
+        <v>624</v>
+      </c>
+      <c r="D9" s="4">
+        <v>2.5</v>
+      </c>
+      <c r="E9" s="5">
+        <v>0</v>
+      </c>
+      <c r="F9" s="5">
+        <v>0</v>
+      </c>
+      <c r="G9" s="5">
+        <v>0</v>
+      </c>
+      <c r="H9" s="5">
+        <v>0</v>
+      </c>
+      <c r="I9" s="5">
+        <v>0</v>
+      </c>
+      <c r="J9" s="5">
+        <v>0</v>
+      </c>
+      <c r="K9" s="5">
+        <v>0</v>
+      </c>
+      <c r="M9" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C10" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="D10" s="4">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="E10" s="4">
+        <v>9</v>
+      </c>
+      <c r="F10" s="4">
+        <v>7.1</v>
+      </c>
+      <c r="G10" s="4">
+        <v>7.75</v>
+      </c>
+      <c r="H10" s="4">
+        <v>7.32</v>
+      </c>
+      <c r="I10" s="4">
+        <v>7.85</v>
+      </c>
+      <c r="J10" s="4">
+        <v>10.63</v>
+      </c>
+      <c r="K10" s="4">
+        <v>10.48</v>
+      </c>
+      <c r="M10" s="4">
+        <v>10.41</v>
+      </c>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C11" s="4" t="s">
+        <v>636</v>
+      </c>
+      <c r="D11" s="4">
+        <v>2</v>
+      </c>
+      <c r="E11" s="4">
+        <v>1.03</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0.97</v>
+      </c>
+      <c r="G11" s="4">
+        <v>1.06</v>
+      </c>
+      <c r="H11" s="4">
+        <v>1.26</v>
+      </c>
+      <c r="I11" s="4">
+        <v>1.18</v>
+      </c>
+      <c r="J11" s="4">
+        <v>1.03</v>
+      </c>
+      <c r="K11" s="4">
+        <v>0.88</v>
+      </c>
+      <c r="M11" s="4">
+        <v>1.28</v>
+      </c>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C12" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="D12" s="4">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="E12" s="4">
+        <v>9.2799999999999994</v>
+      </c>
+      <c r="F12" s="7">
+        <v>6.77</v>
+      </c>
+      <c r="G12" s="4">
+        <v>8.09</v>
+      </c>
+      <c r="H12" s="4">
+        <v>9.2899999999999991</v>
+      </c>
+      <c r="I12" s="4">
+        <v>8.09</v>
+      </c>
+      <c r="J12" s="4">
+        <v>10.41</v>
+      </c>
+      <c r="K12" s="4">
+        <v>9.82</v>
+      </c>
+      <c r="M12" s="4">
+        <v>9.3699999999999992</v>
+      </c>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C13" s="4" t="s">
+        <v>583</v>
+      </c>
+      <c r="D13" s="4">
+        <v>2</v>
+      </c>
+      <c r="E13" s="4">
+        <v>1.25</v>
+      </c>
+      <c r="F13" s="4">
+        <v>1.31</v>
+      </c>
+      <c r="G13" s="4">
+        <v>1.71</v>
+      </c>
+      <c r="H13" s="4">
+        <v>1.41</v>
+      </c>
+      <c r="I13" s="4">
+        <v>1.3</v>
+      </c>
+      <c r="J13" s="4">
+        <v>1.34</v>
+      </c>
+      <c r="K13" s="4">
+        <v>1.32</v>
+      </c>
+      <c r="M13" s="4">
+        <v>1.1499999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C14" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="D14" s="4">
+        <v>12.1</v>
+      </c>
+      <c r="E14" s="4">
+        <v>10.99</v>
+      </c>
+      <c r="F14" s="10">
+        <v>0.79</v>
+      </c>
+      <c r="G14" s="4">
+        <v>7.98</v>
+      </c>
+      <c r="H14" s="10">
+        <v>1.57</v>
+      </c>
+      <c r="I14" s="10">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="J14" s="4">
+        <v>13.74</v>
+      </c>
+      <c r="K14" s="4">
+        <v>10.95</v>
+      </c>
+      <c r="M14" s="4">
+        <v>11.24</v>
+      </c>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C16" s="4" t="s">
+        <v>557</v>
+      </c>
+      <c r="D16" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="E16" s="4">
+        <v>0.06</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>935</v>
+      </c>
+      <c r="G16" s="4">
+        <v>0.03</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>935</v>
+      </c>
+      <c r="I16" s="4">
+        <v>0.09</v>
+      </c>
+      <c r="J16" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="K16" s="4">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="17" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C17" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="D17" s="4">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="E17" s="4">
+        <v>8.15</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>935</v>
+      </c>
+      <c r="G17" s="4">
+        <v>8.77</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>935</v>
+      </c>
+      <c r="I17" s="4">
+        <v>11.46</v>
+      </c>
+      <c r="J17" s="4">
+        <v>8.85</v>
+      </c>
+      <c r="K17" s="4">
+        <v>7.92</v>
+      </c>
+    </row>
+    <row r="18" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C18" s="4" t="s">
+        <v>568</v>
+      </c>
+      <c r="D18" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="E18" s="4">
+        <v>0.12</v>
+      </c>
+      <c r="J18" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C19" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="D19" s="4">
+        <v>9.6</v>
+      </c>
+      <c r="E19" s="4">
+        <v>9.35</v>
+      </c>
+      <c r="J19" s="4">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="K19" s="4">
+        <v>9.15</v>
+      </c>
+    </row>
+    <row r="20" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C20" s="4" t="s">
+        <v>594</v>
+      </c>
+      <c r="D20" s="4">
+        <v>2.1</v>
+      </c>
+      <c r="E20" s="4">
+        <v>1.75</v>
+      </c>
+      <c r="F20" s="5">
+        <v>20.54</v>
+      </c>
+      <c r="G20" s="5">
+        <v>10.47</v>
+      </c>
+      <c r="H20" s="5">
+        <v>21.45</v>
+      </c>
+      <c r="I20" s="5">
+        <v>10.25</v>
+      </c>
+      <c r="J20" s="5">
+        <v>11.11</v>
+      </c>
+      <c r="K20" s="5">
+        <v>11.48</v>
+      </c>
+    </row>
+    <row r="21" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C21" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="D21" s="4">
+        <v>10.1</v>
+      </c>
+      <c r="E21" s="4">
+        <v>11.31</v>
+      </c>
+      <c r="F21" s="5">
+        <v>234.03</v>
+      </c>
+      <c r="G21" s="5">
+        <v>130.13</v>
+      </c>
+      <c r="H21" s="5">
+        <v>276.06</v>
+      </c>
+      <c r="I21" s="5">
+        <v>129.01</v>
+      </c>
+      <c r="J21" s="4">
+        <v>12.03</v>
+      </c>
+      <c r="K21" s="4">
+        <v>11.25</v>
+      </c>
+    </row>
+    <row r="22" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C22" s="4" t="s">
+        <v>624</v>
+      </c>
+      <c r="D22" s="4">
+        <v>2.5</v>
+      </c>
+      <c r="E22" s="4">
+        <v>2.69</v>
+      </c>
+      <c r="F22" s="4">
+        <v>2.54</v>
+      </c>
+      <c r="G22" s="4">
+        <v>1.99</v>
+      </c>
+      <c r="H22" s="4">
+        <v>2.46</v>
+      </c>
+      <c r="I22" s="4">
+        <v>2.23</v>
+      </c>
+      <c r="J22" s="4">
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="K22" s="4">
+        <v>1.91</v>
+      </c>
+    </row>
+    <row r="23" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C23" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="D23" s="4">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="E23" s="4">
+        <v>9.9499999999999993</v>
+      </c>
+      <c r="F23" s="4">
+        <v>10.92</v>
+      </c>
+      <c r="G23" s="4">
+        <v>9.2100000000000009</v>
+      </c>
+      <c r="H23" s="4">
+        <v>10.34</v>
+      </c>
+      <c r="I23" s="4">
+        <v>10.67</v>
+      </c>
+      <c r="J23" s="4">
+        <v>9.4</v>
+      </c>
+      <c r="K23" s="4">
+        <v>10.59</v>
+      </c>
+    </row>
+    <row r="24" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C24" s="4" t="s">
+        <v>636</v>
+      </c>
+      <c r="D24" s="4">
+        <v>2</v>
+      </c>
+      <c r="E24" s="4">
+        <v>1.4</v>
+      </c>
+      <c r="F24" s="4">
+        <v>1.46</v>
+      </c>
+      <c r="G24" s="4">
+        <v>1.31</v>
+      </c>
+      <c r="H24" s="4">
+        <v>1.28</v>
+      </c>
+      <c r="I24" s="4">
+        <v>1.25</v>
+      </c>
+      <c r="J24" s="4">
+        <v>1.21</v>
+      </c>
+      <c r="K24" s="4">
+        <v>1.07</v>
+      </c>
+    </row>
+    <row r="25" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C25" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="D25" s="4">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="E25" s="4">
+        <v>8.99</v>
+      </c>
+      <c r="F25" s="4">
+        <v>7.99</v>
+      </c>
+      <c r="G25" s="4">
+        <v>8.1300000000000008</v>
+      </c>
+      <c r="H25" s="4">
+        <v>7.87</v>
+      </c>
+      <c r="I25" s="4">
+        <v>7.76</v>
+      </c>
+      <c r="J25" s="4">
+        <v>9.16</v>
+      </c>
+      <c r="K25" s="4">
+        <v>9.67</v>
+      </c>
+    </row>
+    <row r="26" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C26" s="4" t="s">
+        <v>583</v>
+      </c>
+      <c r="D26" s="4">
+        <v>2</v>
+      </c>
+      <c r="E26" s="4">
+        <v>1.83</v>
+      </c>
+      <c r="F26" s="4">
+        <v>1.58</v>
+      </c>
+      <c r="G26" s="4">
+        <v>1.84</v>
+      </c>
+      <c r="H26" s="4">
+        <v>1.7</v>
+      </c>
+      <c r="I26" s="4">
+        <v>1.91</v>
+      </c>
+      <c r="J26" s="4">
+        <v>1.87</v>
+      </c>
+      <c r="K26" s="4">
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="27" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C27" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="D27" s="4">
+        <v>12.1</v>
+      </c>
+      <c r="E27" s="4">
+        <v>11.33</v>
+      </c>
+      <c r="F27" s="10">
+        <v>2.5099999999999998</v>
+      </c>
+      <c r="G27" s="4">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="H27" s="7">
+        <v>5.0599999999999996</v>
+      </c>
+      <c r="I27" s="4">
+        <v>10.02</v>
+      </c>
+      <c r="J27" s="4">
+        <v>12.02</v>
+      </c>
+      <c r="K27" s="4">
+        <v>11.13</v>
+      </c>
+    </row>
+    <row r="28" spans="3:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F28" s="9" t="s">
+        <v>936</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2718117C-D7C9-474F-8507-CB4484165567}">
   <dimension ref="A1:BK44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -15105,7 +15931,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{487E77A2-EF46-456E-8204-C18F24ED4825}">
   <dimension ref="A1:BK44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -23554,7 +24380,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD427FA1-9D8B-4207-B0AE-10C3FD99E4EF}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>